<commit_message>
new updated other contact
</commit_message>
<xml_diff>
--- a/utils/reference/bpi_cards_xdays-header.xlsx
+++ b/utils/reference/bpi_cards_xdays-header.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SPM\Documents\XDAYS-AUTOMATION\utils\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58798BD-F8D7-4F9F-B2FA-0F95CB49AC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA16C029-80D1-429A-9266-9745179A7E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$AR$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$AS$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="85">
   <si>
     <t>CUST_ID</t>
   </si>
@@ -280,6 +280,15 @@
   </si>
   <si>
     <t>HO_FLAG</t>
+  </si>
+  <si>
+    <t>OTHER CONTACT</t>
+  </si>
+  <si>
+    <t>OTHER_CONTACT</t>
+  </si>
+  <si>
+    <t>Other contact</t>
   </si>
 </sst>
 </file>
@@ -973,55 +982,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR6"/>
+  <dimension ref="A1:AS6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
-    <col min="8" max="8" width="6.5703125" customWidth="1"/>
-    <col min="9" max="9" width="8.28515625" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" customWidth="1"/>
-    <col min="11" max="11" width="23.5703125" customWidth="1"/>
-    <col min="12" max="12" width="7.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" customWidth="1"/>
-    <col min="15" max="15" width="6.7109375" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" customWidth="1"/>
-    <col min="17" max="17" width="20.85546875" customWidth="1"/>
-    <col min="18" max="18" width="21.7109375" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" customWidth="1"/>
-    <col min="20" max="20" width="28" customWidth="1"/>
-    <col min="21" max="21" width="18.42578125" customWidth="1"/>
-    <col min="22" max="22" width="11.28515625" customWidth="1"/>
-    <col min="23" max="23" width="4.85546875" customWidth="1"/>
-    <col min="24" max="24" width="7.140625" customWidth="1"/>
-    <col min="25" max="25" width="8.7109375" customWidth="1"/>
-    <col min="26" max="26" width="10.7109375" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" customWidth="1"/>
-    <col min="28" max="28" width="12.85546875" customWidth="1"/>
-    <col min="29" max="30" width="12" customWidth="1"/>
-    <col min="31" max="31" width="12.85546875" customWidth="1"/>
-    <col min="32" max="32" width="11.5703125" customWidth="1"/>
-    <col min="33" max="33" width="9.28515625" customWidth="1"/>
-    <col min="34" max="34" width="18.5703125" customWidth="1"/>
-    <col min="35" max="35" width="23" customWidth="1"/>
-    <col min="36" max="36" width="25.28515625" customWidth="1"/>
-    <col min="37" max="37" width="13.28515625" customWidth="1"/>
-    <col min="38" max="38" width="14.5703125" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" customWidth="1"/>
-    <col min="40" max="40" width="8.5703125" customWidth="1"/>
-    <col min="41" max="41" width="9.28515625" customWidth="1"/>
-    <col min="42" max="42" width="9.140625" customWidth="1"/>
-    <col min="43" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="44" width="10.5703125" customWidth="1"/>
+    <col min="5" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.5703125" customWidth="1"/>
+    <col min="13" max="13" width="7.7109375" customWidth="1"/>
+    <col min="14" max="14" width="18.85546875" customWidth="1"/>
+    <col min="15" max="15" width="18.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.7109375" customWidth="1"/>
+    <col min="18" max="18" width="20.85546875" customWidth="1"/>
+    <col min="19" max="19" width="21.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" customWidth="1"/>
+    <col min="21" max="21" width="28" customWidth="1"/>
+    <col min="22" max="22" width="18.42578125" customWidth="1"/>
+    <col min="23" max="23" width="11.28515625" customWidth="1"/>
+    <col min="24" max="24" width="4.85546875" customWidth="1"/>
+    <col min="25" max="25" width="7.140625" customWidth="1"/>
+    <col min="26" max="26" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" customWidth="1"/>
+    <col min="29" max="29" width="12.85546875" customWidth="1"/>
+    <col min="30" max="30" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12" customWidth="1"/>
+    <col min="32" max="32" width="12.85546875" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" customWidth="1"/>
+    <col min="34" max="34" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="18.5703125" customWidth="1"/>
+    <col min="36" max="36" width="23" customWidth="1"/>
+    <col min="37" max="37" width="25.28515625" customWidth="1"/>
+    <col min="38" max="38" width="13.28515625" customWidth="1"/>
+    <col min="39" max="39" width="14.5703125" customWidth="1"/>
+    <col min="40" max="40" width="15.42578125" customWidth="1"/>
+    <col min="41" max="41" width="8.5703125" customWidth="1"/>
+    <col min="42" max="42" width="9.28515625" customWidth="1"/>
+    <col min="43" max="43" width="9.140625" customWidth="1"/>
+    <col min="44" max="44" width="11.42578125" customWidth="1"/>
+    <col min="45" max="45" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1038,124 +1048,127 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="AA1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AF1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="16" t="s">
+      <c r="AG1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="13" t="s">
+      <c r="AJ1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:44">
+    <row r="2" spans="1:45">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1172,124 +1185,127 @@
         <v>4</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="14" t="s">
+      <c r="R2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="U2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="V2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="X2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Z2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="Z2" s="14" t="s">
+      <c r="AA2" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="AA2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AC2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="AD2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AD2" s="5" t="s">
+      <c r="AE2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AE2" s="14" t="s">
+      <c r="AF2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="AF2" s="17" t="s">
+      <c r="AG2" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AG2" s="5" t="s">
+      <c r="AH2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AH2" s="5" t="s">
+      <c r="AI2" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AI2" s="14" t="s">
+      <c r="AJ2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="AJ2" s="5" t="s">
+      <c r="AK2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AK2" s="5" t="s">
+      <c r="AL2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AL2" s="5" t="s">
+      <c r="AM2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="AM2" s="5" t="s">
+      <c r="AN2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AN2" s="5" t="s">
+      <c r="AO2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AO2" s="5" t="s">
+      <c r="AP2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AP2" s="5" t="s">
+      <c r="AQ2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AQ2" s="5" t="s">
+      <c r="AR2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AR2" s="5" t="s">
+      <c r="AS2" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:44">
+    <row r="3" spans="1:45">
       <c r="A3" s="7" t="s">
         <v>44</v>
       </c>
@@ -1303,78 +1319,81 @@
         <v>47</v>
       </c>
       <c r="E3" s="8"/>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="8"/>
+      <c r="K3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="N3" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="P3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="Q3" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" s="15" t="s">
+      <c r="R3" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="T3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="T3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="W3" s="9"/>
       <c r="X3" s="9"/>
-      <c r="Y3" s="9" t="s">
+      <c r="Y3" s="9"/>
+      <c r="Z3" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="Z3" s="9"/>
       <c r="AA3" s="9"/>
-      <c r="AB3" s="9" t="s">
+      <c r="AB3" s="9"/>
+      <c r="AC3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="AC3" s="9" t="s">
+      <c r="AD3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="AE3" s="15" t="s">
+      <c r="AF3" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="AF3" s="9" t="s">
+      <c r="AG3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AH3" t="s">
         <v>76</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="AJ3" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="AK3" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AK3" s="12" t="s">
+      <c r="AL3" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:44">
+    <row r="4" spans="1:45">
       <c r="A4" s="7" t="s">
         <v>44</v>
       </c>
@@ -1388,109 +1407,110 @@
         <v>47</v>
       </c>
       <c r="E4" s="8"/>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8"/>
+      <c r="G4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="8"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="8"/>
+      <c r="K4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="11" t="s">
+      <c r="M4" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>69</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="T4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="T4" s="9" t="s">
+      <c r="U4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V4" s="9" t="s">
+      <c r="W4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="W4" s="9"/>
       <c r="X4" s="9"/>
       <c r="Y4" s="9"/>
       <c r="Z4" s="9"/>
       <c r="AA4" s="9"/>
-      <c r="AB4" s="9" t="s">
+      <c r="AB4" s="9"/>
+      <c r="AC4" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="AC4" s="9" t="s">
+      <c r="AD4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="AE4" s="15" t="s">
+      <c r="AF4" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="AF4" s="9" t="s">
+      <c r="AG4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AI4" s="9" t="s">
+      <c r="AJ4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AJ4" s="9" t="s">
+      <c r="AK4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AK4" s="12" t="s">
+      <c r="AL4" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:44">
+    <row r="5" spans="1:45">
       <c r="A5" s="10" t="s">
         <v>70</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="P5" s="18" t="s">
+      <c r="Q5" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="V5" s="18" t="s">
+      <c r="W5" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>80</v>
       </c>
-      <c r="AF5" s="9" t="s">
+      <c r="AG5" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="AI5" s="9" t="s">
+      <c r="AJ5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="AJ5" s="9" t="s">
+      <c r="AK5" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="AK5" s="9" t="s">
+      <c r="AL5" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:44">
-      <c r="AI6" s="18" t="s">
+    <row r="6" spans="1:45">
+      <c r="AJ6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="AJ6" s="18" t="s">
+      <c r="AK6" s="18" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1498,7 +1518,7 @@
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="8" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:AR1">
+  <conditionalFormatting sqref="A1:AS1">
     <cfRule type="duplicateValues" dxfId="7" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
@@ -1516,10 +1536,10 @@
   <conditionalFormatting sqref="B2:B3">
     <cfRule type="duplicateValues" dxfId="2" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:B3 AS1:XFD1048576 Q4 AF6:AI1048576 AI3:AK3 R3:AG3 C3:P3 R5:AR5 AK6:AR1048576 AP3 C2:AR2 A5:O5">
+  <conditionalFormatting sqref="AT1:XFD1048576 A2:B3 R4 AG6:AJ1048576 AJ3:AL3 S3:AH3 C3:Q3 S5:AS5 AL6:AS1048576 AQ3 C2:AS2 A5:P5">
     <cfRule type="duplicateValues" dxfId="1" priority="29"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:P4 AP4 AI4:AK4 R4:AG4 Q3">
+  <conditionalFormatting sqref="A4:Q4 AQ4 AJ4:AL4 S4:AH4 R3">
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>